<commit_message>
Map 6 and 51 balances are per partner: Rs 1,12,000 and Rs 1,02,400 in all
Total due on land sold is now Rs 19,38,800; after the Rs 20 L token advance MKR
is Rs 61,200 ahead. Summary lines also show the amount per partner.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019SxEhFsRZgodaLxa7Hfpt4
</commit_message>
<xml_diff>
--- a/ledger.xlsx
+++ b/ledger.xlsx
@@ -216,7 +216,7 @@
 Part of Tranche 1 (paid as one lump sum; split here by sq ft sold).</t>
   </si>
   <si>
-    <t xml:space="preserve">₹28,000 balance still to be paid by MKR (per Venu, 17 Oct 2026). The Excel shows the full ₹7,20,000 as received.</t>
+    <t xml:space="preserve">₹28,000 per partner (₹1,12,000 in all) still to be paid by MKR (per Venu, 17 Oct 2026). The Excel shows the full ₹7,20,000 as received.</t>
   </si>
   <si>
     <t xml:space="preserve">33.3XAvg(90, 89,95)</t>
@@ -326,13 +326,13 @@
     <t xml:space="preserve">15XAvg(40,43)</t>
   </si>
   <si>
-    <t xml:space="preserve">₹5,00,000 received against ₹4,97,600 (₹2,400 extra), offset against map 51.</t>
+    <t xml:space="preserve">Excel shows ₹5,00,000 received against ₹4,97,600 owed (₹2,400 extra).</t>
   </si>
   <si>
     <t xml:space="preserve">15XAvg(43,45)</t>
   </si>
   <si>
-    <t xml:space="preserve">₹5,00,000 received against ₹5,28,000 (₹28,000 short). Map 50 received ₹2,400 extra, so ₹25,600 is due across map 50 and 51.</t>
+    <t xml:space="preserve">₹25,600 per partner (₹1,02,400 in all) still to be paid by MKR (per Venu, 17 Oct 2026). The Excel shows ₹5,00,000 received.</t>
   </si>
   <si>
     <t xml:space="preserve">15X45</t>
@@ -1065,7 +1065,7 @@
       </c>
       <c r="B15" s="6" t="n">
         <f aca="false">SUM(Plots!L2:L62)</f>
-        <v>28935200</v>
+        <v>28776800</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="B16" s="7" t="n">
         <f aca="false">B14-B15</f>
-        <v>1780400</v>
+        <v>1938800</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1092,7 +1092,7 @@
       </c>
       <c r="B18" s="7" t="n">
         <f aca="false">B16-B17</f>
-        <v>-219600</v>
+        <v>-61200</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">(B15+B17)/4</f>
-        <v>7733800</v>
+        <v>7694200</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="B22" s="7" t="n">
         <f aca="false">B18/4</f>
-        <v>-54900</v>
+        <v>-15300</v>
       </c>
     </row>
   </sheetData>
@@ -1511,11 +1511,11 @@
         <v>720000</v>
       </c>
       <c r="L7" s="14" t="n">
-        <v>692000</v>
+        <v>608000</v>
       </c>
       <c r="M7" s="13" t="n">
         <f aca="false">K7-N(L7)</f>
-        <v>28000</v>
+        <v>112000</v>
       </c>
       <c r="N7" s="13" t="n">
         <f aca="false">I7*Summary!$B$3</f>
@@ -3848,11 +3848,11 @@
         <v>528000</v>
       </c>
       <c r="L54" s="14" t="n">
-        <v>500000</v>
+        <v>425600</v>
       </c>
       <c r="M54" s="13" t="n">
         <f aca="false">K54-N(L54)</f>
-        <v>28000</v>
+        <v>102400</v>
       </c>
       <c r="N54" s="13" t="n">
         <f aca="false">I54*Summary!$B$3</f>

</xml_diff>

<commit_message>
Ledger: exact areas for map 1, 56 and 59 (no rounding)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019SxEhFsRZgodaLxa7Hfpt4
</commit_message>
<xml_diff>
--- a/ledger.xlsx
+++ b/ledger.xlsx
@@ -1042,7 +1042,7 @@
       </c>
       <c r="B12" s="6" t="n">
         <f aca="false">SUMIFS(Plots!F2:F62,Plots!G2:G62,"Can't be sold")</f>
-        <v>2044.81</v>
+        <v>2044.8125</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1232,7 +1232,7 @@
         <v>10.25</v>
       </c>
       <c r="F2" s="11" t="n">
-        <v>863.56</v>
+        <v>863.5625</v>
       </c>
       <c r="G2" s="9" t="s">
         <v>39</v>
@@ -4079,7 +4079,7 @@
         <v>25.5</v>
       </c>
       <c r="F59" s="11" t="n">
-        <v>745.88</v>
+        <v>745.875</v>
       </c>
       <c r="G59" s="9" t="s">
         <v>49</v>
@@ -4087,7 +4087,7 @@
       <c r="H59" s="11"/>
       <c r="I59" s="12" t="n">
         <f aca="false">IF(G59="Unsold",F59,IF(G59="Part-sold",F59-H59,0))</f>
-        <v>745.88</v>
+        <v>745.875</v>
       </c>
       <c r="J59" s="9"/>
       <c r="K59" s="13" t="n">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="N59" s="13" t="n">
         <f aca="false">I59*Summary!$B$3</f>
-        <v>596704</v>
+        <v>596700</v>
       </c>
       <c r="O59" s="9"/>
       <c r="P59" s="9"/>
@@ -4214,7 +4214,7 @@
         <v>31.5</v>
       </c>
       <c r="F62" s="11" t="n">
-        <v>653.62</v>
+        <v>653.625</v>
       </c>
       <c r="G62" s="9" t="s">
         <v>49</v>
@@ -4222,7 +4222,7 @@
       <c r="H62" s="11"/>
       <c r="I62" s="12" t="n">
         <f aca="false">IF(G62="Unsold",F62,IF(G62="Part-sold",F62-H62,0))</f>
-        <v>653.62</v>
+        <v>653.625</v>
       </c>
       <c r="J62" s="9"/>
       <c r="K62" s="13" t="n">
@@ -4236,7 +4236,7 @@
       </c>
       <c r="N62" s="13" t="n">
         <f aca="false">I62*Summary!$B$3</f>
-        <v>522896</v>
+        <v>522900</v>
       </c>
       <c r="O62" s="9"/>
       <c r="P62" s="9"/>

</xml_diff>